<commit_message>
Rangement OneDrive : sous-dossier CONSTATS, dossier de mission retrouvé, relance du rangement
- Sous-dossier de rangement nommé CONSTATS dans chaque dossier de mission.
- Lien « Ouvrir » du tableau lu sous toutes ses formes (lien web, chemin
  Windows, file:/// codé, chemin relatif au tableau) ; à défaut, dossier
  retrouvé par le n° d'expertise dans le dossier du tableau. Relecture des
  tableaux déjà lus.
- Constat terminé non rangé : motif affiché et bouton « Ranger dans OneDrive ».
- Plus de demande caméra / micro / position après la clôture ou la suppression.
- Titres complets (code du dossier) dans « Sur vos autres appareils ».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VN7zyAzSZYj4G5sqzt6YwG
</commit_message>
<xml_diff>
--- a/tests/fixtures/tableau-cs.xlsx
+++ b/tests/fixtures/tableau-cs.xlsx
@@ -497,9 +497,6 @@
           <t>ICPE</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>Ouvrir</t>
@@ -507,7 +504,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>CS26-002_DELTA</t>
@@ -518,12 +514,6 @@
           <t>Client Delta</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>